<commit_message>
feat: update crawl 14/9
</commit_message>
<xml_diff>
--- a/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
+++ b/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -831,6 +832,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -1004,6 +1006,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="33" t="inlineStr">
         <is>
@@ -8501,24 +8504,48 @@
       </c>
       <c r="B25" s="37" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C25" s="37" t="n"/>
-      <c r="D25" s="90" t="n"/>
-      <c r="E25" s="90" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C25" s="37" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D25" s="90" t="n">
+        <v>46279.01908564815</v>
+      </c>
+      <c r="E25" s="90" t="n">
+        <v>46279.88167824074</v>
+      </c>
       <c r="F25" s="85">
         <f>IF(OR(D25="",E25=""),"",24*(E25-D25))</f>
         <v/>
       </c>
-      <c r="G25" s="86" t="n"/>
-      <c r="H25" s="86" t="n"/>
-      <c r="I25" s="86" t="n"/>
-      <c r="J25" s="86" t="n"/>
-      <c r="K25" s="86" t="n"/>
-      <c r="L25" s="86" t="n"/>
-      <c r="M25" s="86" t="n"/>
-      <c r="N25" s="86" t="n"/>
+      <c r="G25" s="86" t="n">
+        <v>1770</v>
+      </c>
+      <c r="H25" s="86" t="n">
+        <v>1770</v>
+      </c>
+      <c r="I25" s="86" t="n">
+        <v>1654</v>
+      </c>
+      <c r="J25" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="86" t="n">
+        <v>91</v>
+      </c>
+      <c r="L25" s="86" t="n">
+        <v>15</v>
+      </c>
+      <c r="M25" s="86" t="n">
+        <v>10</v>
+      </c>
+      <c r="N25" s="86" t="n">
+        <v>15208</v>
+      </c>
       <c r="O25" s="86" t="n">
         <v>5</v>
       </c>
@@ -8527,7 +8554,11 @@
           <t>vps</t>
         </is>
       </c>
-      <c r="Q25" s="37" t="n"/>
+      <c r="Q25" s="37" t="inlineStr">
+        <is>
+          <t>Run ID 24; deploy https://hotel.projecthub.io.vn/; artifact không lưu; scraper_version 2.3.0; terminal API status completed</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="76" t="n">
@@ -16872,6 +16903,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -17165,6 +17197,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: update crawl 8/10
</commit_message>
<xml_diff>
--- a/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
+++ b/outputs/vps-crawl-planner-20260823/vps_crawl_sampling_master.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -9826,24 +9826,46 @@
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C49" s="13" t="n"/>
-      <c r="D49" s="36" t="n"/>
-      <c r="E49" s="36" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>48</v>
+      </c>
+      <c r="D49" s="36" t="n">
+        <v>46303.02209490741</v>
+      </c>
+      <c r="E49" s="36" t="n">
+        <v>46303.71767361111</v>
+      </c>
       <c r="F49" s="20">
         <f>IF(OR(D49="",E49=""),"",24*(E49-D49))</f>
         <v/>
       </c>
-      <c r="G49" s="22" t="n"/>
-      <c r="H49" s="22" t="n"/>
-      <c r="I49" s="22" t="n"/>
-      <c r="J49" s="22" t="n"/>
-      <c r="K49" s="22" t="n"/>
-      <c r="L49" s="22" t="n"/>
-      <c r="M49" s="22" t="n"/>
-      <c r="N49" s="22" t="n"/>
+      <c r="G49" s="22" t="n">
+        <v>1770</v>
+      </c>
+      <c r="H49" s="22" t="n">
+        <v>1770</v>
+      </c>
+      <c r="I49" s="22" t="n">
+        <v>1503</v>
+      </c>
+      <c r="J49" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="22" t="n">
+        <v>182</v>
+      </c>
+      <c r="L49" s="22" t="n">
+        <v>60</v>
+      </c>
+      <c r="M49" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="N49" s="22" t="n">
+        <v>14523</v>
+      </c>
       <c r="O49" s="22" t="n">
         <v>5</v>
       </c>
@@ -9852,7 +9874,11 @@
           <t>vps</t>
         </is>
       </c>
-      <c r="Q49" s="13" t="n"/>
+      <c r="Q49" s="13" t="inlineStr">
+        <is>
+          <t>Run ID 48; deploy VPS; artifact không lưu; scraper_version 2.3.0</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">

</xml_diff>